<commit_message>
Update year-object reference labels and data.
Refine the reference button/title wording and publish the latest yearobject source updates for deployment.
</commit_message>
<xml_diff>
--- a/yearobject.xlsx
+++ b/yearobject.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="115">
   <si>
     <t>대분류</t>
   </si>
@@ -162,9 +162,6 @@
   </si>
   <si>
     <t>손익계산서 구조 변경 에 따라 全 계열사 계정트리 변경 등 시스템 재무제표 재배치</t>
-  </si>
-  <si>
-    <t>2027년 IFRS19 기준 의무 적용에 따른 대응</t>
   </si>
   <si>
     <t>경영자의 성과측정치(MPM) 도입 장단점 비교 통한 시기 판단</t>
@@ -889,6 +886,9 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <cols>
+    <col customWidth="1" min="2" max="2" width="34.63"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
@@ -1038,10 +1038,10 @@
         <v>42</v>
       </c>
       <c r="B14" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C14" s="6" t="s">
         <v>49</v>
-      </c>
-      <c r="C14" s="6" t="s">
-        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -1074,189 +1074,189 @@
     </row>
     <row r="2">
       <c r="A2" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="B2" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="C2" s="8" t="s">
         <v>52</v>
-      </c>
-      <c r="C2" s="8" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="B3" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="B3" s="8" t="s">
-        <v>52</v>
-      </c>
       <c r="C3" s="8" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="B4" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="B4" s="8" t="s">
-        <v>52</v>
-      </c>
       <c r="C4" s="8" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="B5" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="B5" s="8" t="s">
-        <v>52</v>
-      </c>
       <c r="C5" s="8" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B6" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="C6" s="8" t="s">
         <v>57</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="B8" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="C8" s="8" t="s">
         <v>61</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="B9" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="B9" s="8" t="s">
-        <v>61</v>
-      </c>
       <c r="C9" s="8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="B10" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="B10" s="8" t="s">
-        <v>61</v>
-      </c>
       <c r="C10" s="8" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B11" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="C11" s="8" t="s">
         <v>65</v>
-      </c>
-      <c r="C11" s="8" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="B14" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="C14" s="8" t="s">
         <v>70</v>
-      </c>
-      <c r="C14" s="8" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="B15" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="B15" s="8" t="s">
-        <v>70</v>
-      </c>
       <c r="C15" s="8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B16" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="C16" s="8" t="s">
         <v>73</v>
-      </c>
-      <c r="C16" s="8" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B17" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="C17" s="8" t="s">
         <v>75</v>
-      </c>
-      <c r="C17" s="8" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
   </sheetData>
@@ -1284,189 +1284,189 @@
     </row>
     <row r="2">
       <c r="A2" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="B2" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="C2" s="8" t="s">
         <v>79</v>
-      </c>
-      <c r="C2" s="8" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="B3" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="B3" s="8" t="s">
-        <v>79</v>
-      </c>
       <c r="C3" s="8" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B4" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="C4" s="8" t="s">
         <v>82</v>
-      </c>
-      <c r="C4" s="8" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B6" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="C6" s="8" t="s">
         <v>85</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B8" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="C8" s="8" t="s">
         <v>88</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="B10" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="C10" s="8" t="s">
         <v>92</v>
-      </c>
-      <c r="C10" s="8" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="B11" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="B11" s="8" t="s">
-        <v>92</v>
-      </c>
       <c r="C11" s="8" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B12" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="C12" s="8" t="s">
         <v>95</v>
-      </c>
-      <c r="C12" s="8" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="B14" s="8" t="s">
         <v>98</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="C14" s="8" t="s">
         <v>99</v>
-      </c>
-      <c r="C14" s="8" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="B15" s="8" t="s">
         <v>98</v>
       </c>
-      <c r="B15" s="8" t="s">
-        <v>99</v>
-      </c>
       <c r="C15" s="8" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B16" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="C16" s="8" t="s">
         <v>102</v>
-      </c>
-      <c r="C16" s="8" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B18" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="C18" s="8" t="s">
         <v>105</v>
-      </c>
-      <c r="C18" s="8" t="s">
-        <v>106</v>
       </c>
     </row>
   </sheetData>
@@ -1491,50 +1491,50 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>107</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B4" s="6" t="s">
         <v>110</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B6" s="7" t="s">
         <v>113</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
   </sheetData>

</xml_diff>